<commit_message>
Actualizacion diaria del dashboard de inventarios
</commit_message>
<xml_diff>
--- a/bodegas/001.xlsx
+++ b/bodegas/001.xlsx
@@ -556,10 +556,10 @@
         <v>37</v>
       </c>
       <c r="N4" t="n">
-        <v>27000</v>
+        <v>27021.686746988</v>
       </c>
       <c r="O4" t="n">
-        <v>999000</v>
+        <v>999802.4096385561</v>
       </c>
       <c r="P4" t="n">
         <v>20000</v>
@@ -1466,10 +1466,10 @@
         <v>62</v>
       </c>
       <c r="N27" t="n">
-        <v>14857.623272727</v>
+        <v>14857.623287671</v>
       </c>
       <c r="O27" t="n">
-        <v>921172.642909074</v>
+        <v>921172.643835602</v>
       </c>
       <c r="P27" t="n">
         <v>34900</v>
@@ -4068,10 +4068,10 @@
         <v>873</v>
       </c>
       <c r="N88" t="n">
-        <v>10600</v>
+        <v>10603.665283541</v>
       </c>
       <c r="O88" t="n">
-        <v>9253800</v>
+        <v>9256999.792531293</v>
       </c>
       <c r="P88" t="n">
         <v>17200</v>
@@ -5912,10 +5912,10 @@
         <v>1110</v>
       </c>
       <c r="N129" t="n">
-        <v>4371.1712612367</v>
+        <v>4371.766707533</v>
       </c>
       <c r="O129" t="n">
-        <v>4852000.099972737</v>
+        <v>4852661.04536163</v>
       </c>
       <c r="P129" t="n">
         <v>8900</v>
@@ -7410,10 +7410,10 @@
         <v>36</v>
       </c>
       <c r="N162" t="n">
-        <v>1550.1943880809</v>
+        <v>1550.1943922358</v>
       </c>
       <c r="O162" t="n">
-        <v>55806.99797091239</v>
+        <v>55806.9981204888</v>
       </c>
       <c r="P162" t="n">
         <v>2500</v>
@@ -7623,10 +7623,10 @@
         <v>420</v>
       </c>
       <c r="N167" t="n">
-        <v>2069.4655430712</v>
+        <v>2069.4655178908</v>
       </c>
       <c r="O167" t="n">
-        <v>869175.528089904</v>
+        <v>869175.517514136</v>
       </c>
       <c r="P167" t="n">
         <v>6500</v>
@@ -15754,22 +15754,22 @@
         <v>0</v>
       </c>
       <c r="L348" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M348" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="N348" t="n">
         <v>10219</v>
       </c>
       <c r="O348" t="n">
-        <v>858396</v>
+        <v>756206</v>
       </c>
       <c r="P348" t="n">
         <v>16900</v>
       </c>
       <c r="Q348" t="n">
-        <v>1419600</v>
+        <v>1250600</v>
       </c>
     </row>
     <row r="349">
@@ -16220,10 +16220,10 @@
         <v>839</v>
       </c>
       <c r="N358" t="n">
-        <v>1516.0387548048</v>
+        <v>1516.0387544268</v>
       </c>
       <c r="O358" t="n">
-        <v>1271956.515281227</v>
+        <v>1271956.514964085</v>
       </c>
       <c r="P358" t="n">
         <v>2300</v>
@@ -16444,22 +16444,22 @@
         <v>0</v>
       </c>
       <c r="L363" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M363" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="N363" t="n">
         <v>2327.68</v>
       </c>
       <c r="O363" t="n">
-        <v>39570.56</v>
+        <v>34915.2</v>
       </c>
       <c r="P363" t="n">
         <v>3900</v>
       </c>
       <c r="Q363" t="n">
-        <v>66300</v>
+        <v>58500</v>
       </c>
     </row>
     <row r="364">
@@ -17825,10 +17825,10 @@
         <v>158</v>
       </c>
       <c r="N392" t="n">
-        <v>1690.8700092894</v>
+        <v>1690.870009298</v>
       </c>
       <c r="O392" t="n">
-        <v>267157.4614677252</v>
+        <v>267157.461469084</v>
       </c>
       <c r="P392" t="n">
         <v>3000</v>
@@ -18103,22 +18103,22 @@
         <v>0</v>
       </c>
       <c r="L398" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M398" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="N398" t="n">
-        <v>3907.5003375527</v>
+        <v>3907.5003418803</v>
       </c>
       <c r="O398" t="n">
-        <v>265710.0229535836</v>
+        <v>242265.0211965786</v>
       </c>
       <c r="P398" t="n">
         <v>3900</v>
       </c>
       <c r="Q398" t="n">
-        <v>265200</v>
+        <v>241800</v>
       </c>
     </row>
     <row r="399">

</xml_diff>